<commit_message>
Excel update via Admin Panel
</commit_message>
<xml_diff>
--- a/data/finalDB.xlsx
+++ b/data/finalDB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f-macbook-air/Desktop/2025_mclean/202603_mclean_app/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E169E997-BC19-AA40-AADB-C146DB4ED574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD6F5380-8229-C847-B1E0-5022EE5305D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2214" uniqueCount="1499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2214" uniqueCount="1500">
   <si>
     <t>student_id</t>
   </si>
@@ -4654,6 +4654,10 @@
       </rPr>
       <t>: Excel上で「日付（2026/4/1など）」として認識される形式で入力してください。</t>
     </r>
+  </si>
+  <si>
+    <t>info.furuichi@gmail.com</t>
+    <phoneticPr fontId="10"/>
   </si>
   <si>
     <t>furu3298i@gmail.com</t>
@@ -5332,7 +5336,7 @@
       <c r="T2" s="4"/>
       <c r="U2" s="4"/>
       <c r="V2" s="40" t="s">
-        <v>1498</v>
+        <v>1499</v>
       </c>
       <c r="W2" s="2"/>
       <c r="X2" s="2"/>
@@ -37719,7 +37723,7 @@
   <phoneticPr fontId="10"/>
   <hyperlinks>
     <hyperlink ref="V2" r:id="rId1" xr:uid="{6324563B-CEC5-9542-917B-0889B5498F9E}"/>
-    <hyperlink ref="V3:V112" r:id="rId2" display="furu3298i@gmail.com" xr:uid="{4EB7045B-F14A-B64A-BE47-3DA3A01F305A}"/>
+    <hyperlink ref="V3:V112" r:id="rId2" display="info.furuichi@gmail.com" xr:uid="{74BCB91C-49D1-4443-B65B-F77B70DC90E5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>